<commit_message>
Chart draws at card width (fits 375px); illustrative tag on its own line on phones; XLSX sheet picker for every sheet; layout assertions at 1440/375
</commit_message>
<xml_diff>
--- a/test/fixtures/ramp.xlsx
+++ b/test/fixtures/ramp.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contributors" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort B &amp; notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -568,4 +569,82 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Worker ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Signup Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Vetted On</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Onboarded At</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>First Task Accepted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Ramped At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B-1</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B-2</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>